<commit_message>
BidRadar latest stable version before Mac sync
</commit_message>
<xml_diff>
--- a/bid_results.xlsx
+++ b/bid_results.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V138"/>
+  <dimension ref="A1:V141"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6344,7 +6344,7 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>是</t>
+          <t>否</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
@@ -6422,7 +6422,7 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>是</t>
+          <t>否</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
@@ -6500,7 +6500,7 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>是</t>
+          <t>否</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
@@ -6578,7 +6578,7 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>是</t>
+          <t>否</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
@@ -6656,7 +6656,7 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>是</t>
+          <t>否</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
@@ -6734,7 +6734,7 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>是</t>
+          <t>否</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
@@ -6812,7 +6812,7 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>是</t>
+          <t>否</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
@@ -6890,7 +6890,7 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>是</t>
+          <t>否</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
@@ -6968,7 +6968,7 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>是</t>
+          <t>否</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
@@ -7046,7 +7046,7 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>是</t>
+          <t>否</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
@@ -7124,7 +7124,7 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>是</t>
+          <t>否</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
@@ -7202,7 +7202,7 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>是</t>
+          <t>否</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
@@ -7280,7 +7280,7 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>是</t>
+          <t>否</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
@@ -7358,7 +7358,7 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>是</t>
+          <t>否</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
@@ -7436,7 +7436,7 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>是</t>
+          <t>否</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
@@ -7514,7 +7514,7 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>是</t>
+          <t>否</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
@@ -7592,7 +7592,7 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>是</t>
+          <t>否</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
@@ -7670,7 +7670,7 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>是</t>
+          <t>否</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
@@ -7748,7 +7748,7 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>是</t>
+          <t>否</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
@@ -7826,7 +7826,7 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>是</t>
+          <t>否</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
@@ -7904,7 +7904,7 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>是</t>
+          <t>否</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
@@ -7982,7 +7982,7 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>是</t>
+          <t>否</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
@@ -8060,7 +8060,7 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>是</t>
+          <t>否</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
@@ -8138,7 +8138,7 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>是</t>
+          <t>否</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
@@ -8216,7 +8216,7 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>是</t>
+          <t>否</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
@@ -8294,7 +8294,7 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>是</t>
+          <t>否</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
@@ -8372,7 +8372,7 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>是</t>
+          <t>否</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
@@ -8450,7 +8450,7 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>是</t>
+          <t>否</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
@@ -8528,7 +8528,7 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>是</t>
+          <t>否</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
@@ -8606,7 +8606,7 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>是</t>
+          <t>否</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
@@ -8684,7 +8684,7 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>是</t>
+          <t>否</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
@@ -8762,7 +8762,7 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>是</t>
+          <t>否</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
@@ -8840,7 +8840,7 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>是</t>
+          <t>否</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
@@ -8918,7 +8918,7 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>是</t>
+          <t>否</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
@@ -8996,7 +8996,7 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>是</t>
+          <t>否</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
@@ -9074,7 +9074,7 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>是</t>
+          <t>否</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
@@ -9152,7 +9152,7 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>是</t>
+          <t>否</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
@@ -9230,7 +9230,7 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>是</t>
+          <t>否</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
@@ -9308,7 +9308,7 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>是</t>
+          <t>否</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
@@ -9386,7 +9386,7 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>是</t>
+          <t>否</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
@@ -9464,7 +9464,7 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>是</t>
+          <t>否</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
@@ -9542,7 +9542,7 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>是</t>
+          <t>否</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
@@ -9620,7 +9620,7 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>是</t>
+          <t>否</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
@@ -9698,7 +9698,7 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>是</t>
+          <t>否</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
@@ -9776,7 +9776,7 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>是</t>
+          <t>否</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
@@ -9854,7 +9854,7 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>是</t>
+          <t>否</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
@@ -9932,7 +9932,7 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>是</t>
+          <t>否</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
@@ -10010,7 +10010,7 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>是</t>
+          <t>否</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
@@ -10088,7 +10088,7 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>是</t>
+          <t>否</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
@@ -10166,7 +10166,7 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>是</t>
+          <t>否</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
@@ -10244,7 +10244,7 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>是</t>
+          <t>否</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
@@ -10322,7 +10322,7 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>是</t>
+          <t>否</t>
         </is>
       </c>
       <c r="C123" t="inlineStr">
@@ -10400,7 +10400,7 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>是</t>
+          <t>否</t>
         </is>
       </c>
       <c r="C124" t="inlineStr">
@@ -10478,7 +10478,7 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>是</t>
+          <t>否</t>
         </is>
       </c>
       <c r="C125" t="inlineStr">
@@ -10556,7 +10556,7 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>是</t>
+          <t>否</t>
         </is>
       </c>
       <c r="C126" t="inlineStr">
@@ -10634,7 +10634,7 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>是</t>
+          <t>否</t>
         </is>
       </c>
       <c r="C127" t="inlineStr">
@@ -10712,7 +10712,7 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>是</t>
+          <t>否</t>
         </is>
       </c>
       <c r="C128" t="inlineStr">
@@ -10790,7 +10790,7 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>是</t>
+          <t>否</t>
         </is>
       </c>
       <c r="C129" t="inlineStr">
@@ -10868,7 +10868,7 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>是</t>
+          <t>否</t>
         </is>
       </c>
       <c r="C130" t="inlineStr">
@@ -10946,7 +10946,7 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>是</t>
+          <t>否</t>
         </is>
       </c>
       <c r="C131" t="inlineStr">
@@ -11024,7 +11024,7 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>是</t>
+          <t>否</t>
         </is>
       </c>
       <c r="C132" t="inlineStr">
@@ -11102,7 +11102,7 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>是</t>
+          <t>否</t>
         </is>
       </c>
       <c r="C133" t="inlineStr">
@@ -11180,7 +11180,7 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>是</t>
+          <t>否</t>
         </is>
       </c>
       <c r="C134" t="inlineStr">
@@ -11258,7 +11258,7 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>是</t>
+          <t>否</t>
         </is>
       </c>
       <c r="C135" t="inlineStr">
@@ -11336,7 +11336,7 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>是</t>
+          <t>否</t>
         </is>
       </c>
       <c r="C136" t="inlineStr">
@@ -11414,7 +11414,7 @@
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>是</t>
+          <t>否</t>
         </is>
       </c>
       <c r="C137" t="inlineStr">
@@ -11492,7 +11492,7 @@
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>是</t>
+          <t>否</t>
         </is>
       </c>
       <c r="C138" t="inlineStr">
@@ -11562,6 +11562,256 @@
         </is>
       </c>
     </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>link:javascript:urlOpen('8a9c96a69f26595d019f26a3b282174d')</t>
+        </is>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="C139" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="D139" t="inlineStr">
+        <is>
+          <t>纸箱</t>
+        </is>
+      </c>
+      <c r="E139" t="inlineStr"/>
+      <c r="F139" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="G139" t="inlineStr"/>
+      <c r="H139" t="inlineStr">
+        <is>
+          <t>广源公司采购纸箱项目公开招标公告</t>
+        </is>
+      </c>
+      <c r="I139" t="inlineStr"/>
+      <c r="J139" t="inlineStr"/>
+      <c r="K139" t="inlineStr"/>
+      <c r="L139" t="inlineStr"/>
+      <c r="M139" t="inlineStr"/>
+      <c r="N139" t="inlineStr">
+        <is>
+          <t>中国招标投标公共服务平台公开搜索页</t>
+        </is>
+      </c>
+      <c r="O139" t="inlineStr">
+        <is>
+          <t>javascript:urlOpen('8a9c96a69f26595d019f26a3b282174d')</t>
+        </is>
+      </c>
+      <c r="P139" t="inlineStr">
+        <is>
+          <t>纸箱</t>
+        </is>
+      </c>
+      <c r="Q139" t="n">
+        <v>0</v>
+      </c>
+      <c r="R139" t="inlineStr">
+        <is>
+          <t>★</t>
+        </is>
+      </c>
+      <c r="S139" t="inlineStr">
+        <is>
+          <t>暂不优先</t>
+        </is>
+      </c>
+      <c r="T139" t="inlineStr">
+        <is>
+          <t>观察</t>
+        </is>
+      </c>
+      <c r="U139" t="inlineStr">
+        <is>
+          <t>待跟进</t>
+        </is>
+      </c>
+      <c r="V139" t="inlineStr">
+        <is>
+          <t>公开网页采集</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>link:javascript:urlOpen('244b17b6d3b54e829d5a752307a38ea4')</t>
+        </is>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="C140" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="D140" t="inlineStr">
+        <is>
+          <t>瓦楞纸箱</t>
+        </is>
+      </c>
+      <c r="E140" t="inlineStr"/>
+      <c r="F140" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="G140" t="inlineStr"/>
+      <c r="H140" t="inlineStr">
+        <is>
+          <t>福建省三明金叶复烤有限公司瓦楞纸箱采购项目-公开招标公告</t>
+        </is>
+      </c>
+      <c r="I140" t="inlineStr"/>
+      <c r="J140" t="inlineStr"/>
+      <c r="K140" t="inlineStr"/>
+      <c r="L140" t="inlineStr"/>
+      <c r="M140" t="inlineStr"/>
+      <c r="N140" t="inlineStr">
+        <is>
+          <t>中国招标投标公共服务平台公开搜索页</t>
+        </is>
+      </c>
+      <c r="O140" t="inlineStr">
+        <is>
+          <t>javascript:urlOpen('244b17b6d3b54e829d5a752307a38ea4')</t>
+        </is>
+      </c>
+      <c r="P140" t="inlineStr">
+        <is>
+          <t>纸箱、瓦楞纸箱</t>
+        </is>
+      </c>
+      <c r="Q140" t="n">
+        <v>0</v>
+      </c>
+      <c r="R140" t="inlineStr">
+        <is>
+          <t>★</t>
+        </is>
+      </c>
+      <c r="S140" t="inlineStr">
+        <is>
+          <t>暂不优先</t>
+        </is>
+      </c>
+      <c r="T140" t="inlineStr">
+        <is>
+          <t>观察</t>
+        </is>
+      </c>
+      <c r="U140" t="inlineStr">
+        <is>
+          <t>待跟进</t>
+        </is>
+      </c>
+      <c r="V140" t="inlineStr">
+        <is>
+          <t>公开网页采集</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>link:javascript:urlOpen('6899db097d18418fb327dbd5ff77c854')</t>
+        </is>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="C141" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="D141" t="inlineStr">
+        <is>
+          <t>瓦楞纸箱</t>
+        </is>
+      </c>
+      <c r="E141" t="inlineStr">
+        <is>
+          <t>山东</t>
+        </is>
+      </c>
+      <c r="F141" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="G141" t="inlineStr"/>
+      <c r="H141" t="inlineStr">
+        <is>
+          <t>山东福瑞达生物股份、明仁福瑞达瓦楞包装箱项目竞争性磋商公告</t>
+        </is>
+      </c>
+      <c r="I141" t="inlineStr"/>
+      <c r="J141" t="inlineStr"/>
+      <c r="K141" t="inlineStr"/>
+      <c r="L141" t="inlineStr"/>
+      <c r="M141" t="inlineStr"/>
+      <c r="N141" t="inlineStr">
+        <is>
+          <t>中国招标投标公共服务平台公开搜索页</t>
+        </is>
+      </c>
+      <c r="O141" t="inlineStr">
+        <is>
+          <t>javascript:urlOpen('6899db097d18418fb327dbd5ff77c854')</t>
+        </is>
+      </c>
+      <c r="P141" t="inlineStr">
+        <is>
+          <t>包装箱</t>
+        </is>
+      </c>
+      <c r="Q141" t="n">
+        <v>0</v>
+      </c>
+      <c r="R141" t="inlineStr">
+        <is>
+          <t>★</t>
+        </is>
+      </c>
+      <c r="S141" t="inlineStr">
+        <is>
+          <t>暂不优先</t>
+        </is>
+      </c>
+      <c r="T141" t="inlineStr">
+        <is>
+          <t>观察</t>
+        </is>
+      </c>
+      <c r="U141" t="inlineStr">
+        <is>
+          <t>待跟进</t>
+        </is>
+      </c>
+      <c r="V141" t="inlineStr">
+        <is>
+          <t>公开网页采集</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>